<commit_message>
style: translate country names to Turkish in database and Excel
</commit_message>
<xml_diff>
--- a/fuardan firma bulma/Robotsepeti_Tum_Fuar_Listesi_BirlestikOtomatik.xlsx
+++ b/fuardan firma bulma/Robotsepeti_Tum_Fuar_Listesi_BirlestikOtomatik.xlsx
@@ -5533,7 +5533,7 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -5593,7 +5593,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Tayvan</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -5653,7 +5653,7 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -5713,7 +5713,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -5773,7 +5773,7 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -5833,7 +5833,7 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -6013,7 +6013,7 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Tayvan</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -6073,7 +6073,7 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -6193,7 +6193,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -6253,7 +6253,7 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Avusturya</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -6313,7 +6313,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -6373,7 +6373,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>İngiltere</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -6493,7 +6493,7 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -6553,7 +6553,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -6673,7 +6673,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -6733,7 +6733,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -6793,7 +6793,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -6913,7 +6913,7 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -6973,7 +6973,7 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -7033,7 +7033,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -7153,7 +7153,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -7213,7 +7213,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -7273,7 +7273,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -7393,7 +7393,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -7453,7 +7453,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -7513,7 +7513,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -7573,7 +7573,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -7633,7 +7633,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -7693,7 +7693,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -7753,7 +7753,7 @@
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Belçika</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
@@ -7813,7 +7813,7 @@
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Portekiz</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
@@ -7993,7 +7993,7 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Singapur</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
@@ -8113,7 +8113,7 @@
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
@@ -8173,7 +8173,7 @@
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
@@ -8233,7 +8233,7 @@
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
@@ -8293,7 +8293,7 @@
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
@@ -8353,7 +8353,7 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -8413,7 +8413,7 @@
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -8533,7 +8533,7 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -8593,7 +8593,7 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -8653,7 +8653,7 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -8713,7 +8713,7 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -8773,7 +8773,7 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -8833,7 +8833,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -8954,7 +8954,7 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -9074,7 +9074,7 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Avusturya</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -9134,7 +9134,7 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -9194,7 +9194,7 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -9254,7 +9254,7 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Portekiz</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -9374,7 +9374,7 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Kanada</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -9434,7 +9434,7 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -9494,7 +9494,7 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -9554,7 +9554,7 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Belçika</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -9666,7 +9666,7 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -9726,7 +9726,7 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Slovenya</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -9786,7 +9786,7 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -9846,7 +9846,7 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -9906,7 +9906,7 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -9966,7 +9966,7 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -10018,7 +10018,7 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Belçika</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -10078,7 +10078,7 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -10138,7 +10138,7 @@
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
@@ -10198,7 +10198,7 @@
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
@@ -10258,7 +10258,7 @@
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -10318,7 +10318,7 @@
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Kanada</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
@@ -10378,7 +10378,7 @@
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -10498,7 +10498,7 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>United States of America</t>
+          <t>ABD</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -10618,7 +10618,7 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -10678,7 +10678,7 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Tayvan</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -10738,7 +10738,7 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Hollanda</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -10798,7 +10798,7 @@
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
@@ -10858,7 +10858,7 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -10918,7 +10918,7 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -10978,7 +10978,7 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
@@ -11038,7 +11038,7 @@
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Hollanda</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
@@ -11098,7 +11098,7 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
@@ -11158,7 +11158,7 @@
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
@@ -11218,7 +11218,7 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Belçika</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -11278,7 +11278,7 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -11458,7 +11458,7 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
@@ -11518,7 +11518,7 @@
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -11578,7 +11578,7 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
@@ -11638,7 +11638,7 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
@@ -11698,7 +11698,7 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -11758,7 +11758,7 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
@@ -11818,7 +11818,7 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
@@ -11878,7 +11878,7 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
@@ -11938,7 +11938,7 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
@@ -11998,7 +11998,7 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
@@ -12058,7 +12058,7 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -12118,7 +12118,7 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
@@ -12178,7 +12178,7 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>İsrail</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -12238,7 +12238,7 @@
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>United States of America</t>
+          <t>ABD</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
@@ -12298,7 +12298,7 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
@@ -12538,7 +12538,7 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Belçika</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
@@ -12598,7 +12598,7 @@
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
@@ -12658,7 +12658,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -12718,7 +12718,7 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Portekiz</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
@@ -12778,7 +12778,7 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Singapur</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -12838,7 +12838,7 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
@@ -12898,7 +12898,7 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -12958,7 +12958,7 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
@@ -13018,7 +13018,7 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -13078,7 +13078,7 @@
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -13138,7 +13138,7 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -13198,7 +13198,7 @@
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -13258,7 +13258,7 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -13378,7 +13378,7 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -13438,7 +13438,7 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -13618,7 +13618,7 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>İspanya</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -13678,7 +13678,7 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -13738,7 +13738,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -13798,7 +13798,7 @@
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -13858,7 +13858,7 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -13978,7 +13978,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -14038,7 +14038,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Slovenya</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -14098,7 +14098,7 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -14158,7 +14158,7 @@
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Kanada</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -14218,7 +14218,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -14278,7 +14278,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -14338,7 +14338,7 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -14458,7 +14458,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -14578,7 +14578,7 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -14638,7 +14638,7 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>United States of America</t>
+          <t>ABD</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -14698,7 +14698,7 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -14758,7 +14758,7 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -14818,7 +14818,7 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Japonya</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -14878,7 +14878,7 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
@@ -14938,7 +14938,7 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -14998,7 +14998,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -15058,7 +15058,7 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
@@ -15118,7 +15118,7 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -15178,7 +15178,7 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
@@ -15238,7 +15238,7 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -15298,7 +15298,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Tayvan</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -15358,7 +15358,7 @@
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -15410,7 +15410,7 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -15470,7 +15470,7 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -15530,7 +15530,7 @@
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -15590,7 +15590,7 @@
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -15650,7 +15650,7 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -15710,7 +15710,7 @@
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
@@ -15770,7 +15770,7 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Tayvan</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -15830,7 +15830,7 @@
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -15890,7 +15890,7 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -15950,7 +15950,7 @@
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
@@ -16070,7 +16070,7 @@
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
@@ -16130,7 +16130,7 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -16190,7 +16190,7 @@
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
@@ -16250,7 +16250,7 @@
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
@@ -16310,7 +16310,7 @@
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Tayvan</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
@@ -16370,7 +16370,7 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -16430,7 +16430,7 @@
       </c>
       <c r="C267" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
@@ -16490,7 +16490,7 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -16550,7 +16550,7 @@
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
@@ -16610,7 +16610,7 @@
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
@@ -16670,7 +16670,7 @@
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Kanada</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
@@ -16730,7 +16730,7 @@
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
@@ -16850,7 +16850,7 @@
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
@@ -16910,7 +16910,7 @@
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Kanada</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -16970,7 +16970,7 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Kanada</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
@@ -17030,7 +17030,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Japonya</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -17090,7 +17090,7 @@
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
@@ -17150,7 +17150,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -17210,7 +17210,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -17270,7 +17270,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -17450,7 +17450,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -17510,7 +17510,7 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -17570,7 +17570,7 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -17630,7 +17630,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -17682,7 +17682,7 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -17742,7 +17742,7 @@
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
@@ -17802,7 +17802,7 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
@@ -17862,7 +17862,7 @@
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
@@ -17922,7 +17922,7 @@
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -18042,7 +18042,7 @@
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
@@ -18102,7 +18102,7 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -18162,7 +18162,7 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
@@ -18222,7 +18222,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -18282,7 +18282,7 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
@@ -18342,7 +18342,7 @@
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
@@ -18402,7 +18402,7 @@
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
@@ -18462,7 +18462,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -18522,7 +18522,7 @@
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
@@ -18582,7 +18582,7 @@
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Tayvan</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr">
@@ -18642,7 +18642,7 @@
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
@@ -18702,7 +18702,7 @@
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Çekya</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr">
@@ -18762,7 +18762,7 @@
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
@@ -20142,7 +20142,7 @@
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>Korea</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D329" s="2" t="inlineStr">
@@ -33147,7 +33147,7 @@
       </c>
       <c r="C548" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D548" s="2" t="inlineStr">
@@ -51691,7 +51691,7 @@
       </c>
       <c r="C873" s="2" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Belçika</t>
         </is>
       </c>
       <c r="D873" s="2" t="inlineStr">
@@ -51751,7 +51751,7 @@
       </c>
       <c r="C874" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D874" s="2" t="inlineStr">
@@ -51871,7 +51871,7 @@
       </c>
       <c r="C876" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Kanada</t>
         </is>
       </c>
       <c r="D876" s="2" t="inlineStr">
@@ -51931,7 +51931,7 @@
       </c>
       <c r="C877" s="2" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>İsrail</t>
         </is>
       </c>
       <c r="D877" s="2" t="inlineStr">
@@ -51991,7 +51991,7 @@
       </c>
       <c r="C878" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D878" s="2" t="inlineStr">
@@ -52051,7 +52051,7 @@
       </c>
       <c r="C879" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D879" s="2" t="inlineStr">
@@ -52111,7 +52111,7 @@
       </c>
       <c r="C880" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D880" s="2" t="inlineStr">
@@ -52171,7 +52171,7 @@
       </c>
       <c r="C881" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D881" s="2" t="inlineStr">
@@ -52231,7 +52231,7 @@
       </c>
       <c r="C882" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D882" s="2" t="inlineStr">
@@ -52291,7 +52291,7 @@
       </c>
       <c r="C883" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D883" s="2" t="inlineStr">
@@ -52351,7 +52351,7 @@
       </c>
       <c r="C884" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D884" s="2" t="inlineStr">
@@ -52411,7 +52411,7 @@
       </c>
       <c r="C885" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D885" s="2" t="inlineStr">
@@ -52471,7 +52471,7 @@
       </c>
       <c r="C886" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D886" s="2" t="inlineStr">
@@ -52531,7 +52531,7 @@
       </c>
       <c r="C887" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D887" s="2" t="inlineStr">
@@ -52591,7 +52591,7 @@
       </c>
       <c r="C888" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Avusturya</t>
         </is>
       </c>
       <c r="D888" s="2" t="inlineStr">
@@ -52651,7 +52651,7 @@
       </c>
       <c r="C889" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D889" s="2" t="inlineStr">
@@ -52711,7 +52711,7 @@
       </c>
       <c r="C890" s="2" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Japonya</t>
         </is>
       </c>
       <c r="D890" s="2" t="inlineStr">
@@ -52771,7 +52771,7 @@
       </c>
       <c r="C891" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D891" s="2" t="inlineStr">
@@ -52891,7 +52891,7 @@
       </c>
       <c r="C893" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D893" s="2" t="inlineStr">
@@ -52951,7 +52951,7 @@
       </c>
       <c r="C894" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D894" s="2" t="inlineStr">
@@ -53011,7 +53011,7 @@
       </c>
       <c r="C895" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Kanada</t>
         </is>
       </c>
       <c r="D895" s="2" t="inlineStr">
@@ -53071,7 +53071,7 @@
       </c>
       <c r="C896" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D896" s="2" t="inlineStr">
@@ -53131,7 +53131,7 @@
       </c>
       <c r="C897" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D897" s="2" t="inlineStr">
@@ -53191,7 +53191,7 @@
       </c>
       <c r="C898" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D898" s="2" t="inlineStr">
@@ -53251,7 +53251,7 @@
       </c>
       <c r="C899" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>İsveç</t>
         </is>
       </c>
       <c r="D899" s="2" t="inlineStr">
@@ -53311,7 +53311,7 @@
       </c>
       <c r="C900" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Portekiz</t>
         </is>
       </c>
       <c r="D900" s="2" t="inlineStr">
@@ -53371,7 +53371,7 @@
       </c>
       <c r="C901" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D901" s="2" t="inlineStr">
@@ -53431,7 +53431,7 @@
       </c>
       <c r="C902" s="2" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>İsviçre</t>
         </is>
       </c>
       <c r="D902" s="2" t="inlineStr">
@@ -53491,7 +53491,7 @@
       </c>
       <c r="C903" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D903" s="2" t="inlineStr">
@@ -53551,7 +53551,7 @@
       </c>
       <c r="C904" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D904" s="2" t="inlineStr">
@@ -53611,7 +53611,7 @@
       </c>
       <c r="C905" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D905" s="2" t="inlineStr">
@@ -53671,7 +53671,7 @@
       </c>
       <c r="C906" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Avusturya</t>
         </is>
       </c>
       <c r="D906" s="2" t="inlineStr">
@@ -53731,7 +53731,7 @@
       </c>
       <c r="C907" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D907" s="2" t="inlineStr">
@@ -53791,7 +53791,7 @@
       </c>
       <c r="C908" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D908" s="2" t="inlineStr">
@@ -53851,7 +53851,7 @@
       </c>
       <c r="C909" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D909" s="2" t="inlineStr">
@@ -53911,7 +53911,7 @@
       </c>
       <c r="C910" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D910" s="2" t="inlineStr">
@@ -53971,7 +53971,7 @@
       </c>
       <c r="C911" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D911" s="2" t="inlineStr">
@@ -54031,7 +54031,7 @@
       </c>
       <c r="C912" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D912" s="2" t="inlineStr">
@@ -54091,7 +54091,7 @@
       </c>
       <c r="C913" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D913" s="2" t="inlineStr">
@@ -54151,7 +54151,7 @@
       </c>
       <c r="C914" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D914" s="2" t="inlineStr">
@@ -54211,7 +54211,7 @@
       </c>
       <c r="C915" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D915" s="2" t="inlineStr">
@@ -54327,7 +54327,7 @@
       </c>
       <c r="C917" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D917" s="2" t="inlineStr">
@@ -54387,7 +54387,7 @@
       </c>
       <c r="C918" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Kanada</t>
         </is>
       </c>
       <c r="D918" s="2" t="inlineStr">
@@ -54447,7 +54447,7 @@
       </c>
       <c r="C919" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D919" s="2" t="inlineStr">
@@ -54507,7 +54507,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -54567,7 +54567,7 @@
       </c>
       <c r="C921" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Portekiz</t>
         </is>
       </c>
       <c r="D921" s="2" t="inlineStr">
@@ -54627,7 +54627,7 @@
       </c>
       <c r="C922" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Avusturya</t>
         </is>
       </c>
       <c r="D922" s="2" t="inlineStr">
@@ -54687,7 +54687,7 @@
       </c>
       <c r="C923" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D923" s="2" t="inlineStr">
@@ -54747,7 +54747,7 @@
       </c>
       <c r="C924" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D924" s="2" t="inlineStr">
@@ -54803,7 +54803,7 @@
       </c>
       <c r="C925" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D925" s="2" t="inlineStr">
@@ -54863,7 +54863,7 @@
       </c>
       <c r="C926" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D926" s="2" t="inlineStr">
@@ -54923,7 +54923,7 @@
       </c>
       <c r="C927" s="2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Hollanda</t>
         </is>
       </c>
       <c r="D927" s="2" t="inlineStr">
@@ -54983,7 +54983,7 @@
       </c>
       <c r="C928" s="2" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Finlandiya</t>
         </is>
       </c>
       <c r="D928" s="2" t="inlineStr">
@@ -55043,7 +55043,7 @@
       </c>
       <c r="C929" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Kanada</t>
         </is>
       </c>
       <c r="D929" s="2" t="inlineStr">
@@ -55103,7 +55103,7 @@
       </c>
       <c r="C930" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D930" s="2" t="inlineStr">
@@ -55163,7 +55163,7 @@
       </c>
       <c r="C931" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Portekiz</t>
         </is>
       </c>
       <c r="D931" s="2" t="inlineStr">
@@ -55223,7 +55223,7 @@
       </c>
       <c r="C932" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D932" s="2" t="inlineStr">
@@ -55283,7 +55283,7 @@
       </c>
       <c r="C933" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D933" s="2" t="inlineStr">
@@ -55343,7 +55343,7 @@
       </c>
       <c r="C934" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Portekiz</t>
         </is>
       </c>
       <c r="D934" s="2" t="inlineStr">
@@ -55403,7 +55403,7 @@
       </c>
       <c r="C935" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D935" s="2" t="inlineStr">
@@ -55463,7 +55463,7 @@
       </c>
       <c r="C936" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Avusturya</t>
         </is>
       </c>
       <c r="D936" s="2" t="inlineStr">
@@ -55523,7 +55523,7 @@
       </c>
       <c r="C937" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D937" s="2" t="inlineStr">
@@ -55583,7 +55583,7 @@
       </c>
       <c r="C938" s="2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Hollanda</t>
         </is>
       </c>
       <c r="D938" s="2" t="inlineStr">
@@ -55643,7 +55643,7 @@
       </c>
       <c r="C939" s="2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Hollanda</t>
         </is>
       </c>
       <c r="D939" s="2" t="inlineStr">
@@ -55703,7 +55703,7 @@
       </c>
       <c r="C940" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D940" s="2" t="inlineStr">
@@ -55763,7 +55763,7 @@
       </c>
       <c r="C941" s="2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Hollanda</t>
         </is>
       </c>
       <c r="D941" s="2" t="inlineStr">
@@ -55823,7 +55823,7 @@
       </c>
       <c r="C942" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D942" s="2" t="inlineStr">
@@ -55879,7 +55879,7 @@
       </c>
       <c r="C943" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D943" s="2" t="inlineStr">
@@ -55935,7 +55935,7 @@
       </c>
       <c r="C944" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Portekiz</t>
         </is>
       </c>
       <c r="D944" s="2" t="inlineStr">
@@ -55995,7 +55995,7 @@
       </c>
       <c r="C945" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Avusturya</t>
         </is>
       </c>
       <c r="D945" s="2" t="inlineStr">
@@ -56055,7 +56055,7 @@
       </c>
       <c r="C946" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Kanada</t>
         </is>
       </c>
       <c r="D946" s="2" t="inlineStr">
@@ -56115,7 +56115,7 @@
       </c>
       <c r="C947" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D947" s="2" t="inlineStr">
@@ -56175,7 +56175,7 @@
       </c>
       <c r="C948" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Fransa</t>
         </is>
       </c>
       <c r="D948" s="2" t="inlineStr">
@@ -56235,7 +56235,7 @@
       </c>
       <c r="C949" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D949" s="2" t="inlineStr">
@@ -56295,7 +56295,7 @@
       </c>
       <c r="C950" s="2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Hollanda</t>
         </is>
       </c>
       <c r="D950" s="2" t="inlineStr">
@@ -56355,7 +56355,7 @@
       </c>
       <c r="C951" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D951" s="2" t="inlineStr">
@@ -56415,7 +56415,7 @@
       </c>
       <c r="C952" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D952" s="2" t="inlineStr">
@@ -56471,7 +56471,7 @@
       </c>
       <c r="C953" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D953" s="2" t="inlineStr">
@@ -56531,7 +56531,7 @@
       </c>
       <c r="C954" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D954" s="2" t="inlineStr">
@@ -56591,7 +56591,7 @@
       </c>
       <c r="C955" s="2" t="inlineStr">
         <is>
-          <t>Taiwan (Chinese Taipei)</t>
+          <t>Tayvan</t>
         </is>
       </c>
       <c r="D955" s="2" t="inlineStr">
@@ -56651,7 +56651,7 @@
       </c>
       <c r="C956" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Avusturya</t>
         </is>
       </c>
       <c r="D956" s="2" t="inlineStr">
@@ -56711,7 +56711,7 @@
       </c>
       <c r="C957" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D957" s="2" t="inlineStr">
@@ -56771,7 +56771,7 @@
       </c>
       <c r="C958" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Güney Kore</t>
         </is>
       </c>
       <c r="D958" s="2" t="inlineStr">
@@ -56827,7 +56827,7 @@
       </c>
       <c r="C959" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D959" s="2" t="inlineStr">
@@ -56947,7 +56947,7 @@
       </c>
       <c r="C961" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D961" s="2" t="inlineStr">
@@ -57007,7 +57007,7 @@
       </c>
       <c r="C962" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D962" s="2" t="inlineStr">
@@ -57067,7 +57067,7 @@
       </c>
       <c r="C963" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D963" s="2" t="inlineStr">
@@ -57127,7 +57127,7 @@
       </c>
       <c r="C964" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Avusturya</t>
         </is>
       </c>
       <c r="D964" s="2" t="inlineStr">
@@ -57187,7 +57187,7 @@
       </c>
       <c r="C965" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D965" s="2" t="inlineStr">
@@ -57247,7 +57247,7 @@
       </c>
       <c r="C966" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Portekiz</t>
         </is>
       </c>
       <c r="D966" s="2" t="inlineStr">
@@ -57307,7 +57307,7 @@
       </c>
       <c r="C967" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D967" s="2" t="inlineStr">
@@ -57367,7 +57367,7 @@
       </c>
       <c r="C968" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D968" s="2" t="inlineStr">
@@ -57427,7 +57427,7 @@
       </c>
       <c r="C969" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D969" s="2" t="inlineStr">
@@ -57483,7 +57483,7 @@
       </c>
       <c r="C970" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D970" s="2" t="inlineStr">
@@ -57543,7 +57543,7 @@
       </c>
       <c r="C971" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Avusturya</t>
         </is>
       </c>
       <c r="D971" s="2" t="inlineStr">
@@ -57603,7 +57603,7 @@
       </c>
       <c r="C972" s="2" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Portekiz</t>
         </is>
       </c>
       <c r="D972" s="2" t="inlineStr">
@@ -57663,7 +57663,7 @@
       </c>
       <c r="C973" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D973" s="2" t="inlineStr">
@@ -57723,7 +57723,7 @@
       </c>
       <c r="C974" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>İtalya</t>
         </is>
       </c>
       <c r="D974" s="2" t="inlineStr">
@@ -57783,7 +57783,7 @@
       </c>
       <c r="C975" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D975" s="2" t="inlineStr">
@@ -57843,7 +57843,7 @@
       </c>
       <c r="C976" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>İspanya</t>
         </is>
       </c>
       <c r="D976" s="2" t="inlineStr">
@@ -57903,7 +57903,7 @@
       </c>
       <c r="C977" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Fransa</t>
         </is>
       </c>
       <c r="D977" s="2" t="inlineStr">
@@ -58023,7 +58023,7 @@
       </c>
       <c r="C979" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D979" s="2" t="inlineStr">
@@ -58083,7 +58083,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>İsrail</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr">
@@ -58143,7 +58143,7 @@
       </c>
       <c r="C981" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Avusturya</t>
         </is>
       </c>
       <c r="D981" s="2" t="inlineStr">
@@ -58203,7 +58203,7 @@
       </c>
       <c r="C982" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Almanya</t>
         </is>
       </c>
       <c r="D982" s="2" t="inlineStr">
@@ -58263,7 +58263,7 @@
       </c>
       <c r="C983" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D983" s="2" t="inlineStr">
@@ -58323,7 +58323,7 @@
       </c>
       <c r="C984" s="2" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Avusturya</t>
         </is>
       </c>
       <c r="D984" s="2" t="inlineStr">
@@ -58383,7 +58383,7 @@
       </c>
       <c r="C985" s="2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Hollanda</t>
         </is>
       </c>
       <c r="D985" s="2" t="inlineStr">
@@ -58443,7 +58443,7 @@
       </c>
       <c r="C986" s="2" t="inlineStr">
         <is>
-          <t>Taiwan (Chinese Taipei)</t>
+          <t>Tayvan</t>
         </is>
       </c>
       <c r="D986" s="2" t="inlineStr">
@@ -58503,7 +58503,7 @@
       </c>
       <c r="C987" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Çin</t>
         </is>
       </c>
       <c r="D987" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add qualified leads from Expopharm 2025 and update Excel/JS database
</commit_message>
<xml_diff>
--- a/fuardan firma bulma/Robotsepeti_Tum_Fuar_Listesi_BirlestikOtomatik.xlsx
+++ b/fuardan firma bulma/Robotsepeti_Tum_Fuar_Listesi_BirlestikOtomatik.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Fuar Katılımcı Listesi" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fuar Katılımcı Listesi'!$A$1:$L$987</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fuar Katılımcı Listesi'!$A$1:$L$1000</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L987"/>
+  <dimension ref="A1:L1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -58552,8 +58552,736 @@
         </is>
       </c>
     </row>
+    <row r="988">
+      <c r="A988" s="2" t="n">
+        <v>987</v>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> alphacheck -Diabetes Hilfsmittel mit Konzept- CareSens Air CGMS - Berger Med GmbH</t>
+        </is>
+      </c>
+      <c r="C988" s="2" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="D988" s="2" t="inlineStr"/>
+      <c r="E988" s="2" t="inlineStr">
+        <is>
+          <t>A2 - E1</t>
+        </is>
+      </c>
+      <c r="F988" t="inlineStr">
+        <is>
+          <t>Medikal / Hassas Talaşlı İmalat</t>
+        </is>
+      </c>
+      <c r="G988" t="inlineStr">
+        <is>
+          <t>EXPOPHARM 2025</t>
+        </is>
+      </c>
+      <c r="H988" t="inlineStr">
+        <is>
+          <t>http://www.bergermed.de</t>
+        </is>
+      </c>
+      <c r="I988" t="inlineStr">
+        <is>
+          <t>Tel: 00496441897730</t>
+        </is>
+      </c>
+      <c r="J988" s="6" t="inlineStr">
+        <is>
+          <t>Yüksek Öncelik</t>
+        </is>
+      </c>
+      <c r="K988" s="4" t="inlineStr">
+        <is>
+          <t>Hassas iğne, sprey valfleri, insülin kalem iğneleri, lansetler veya ilaç dozaj kovanları üreten, optik metroloji tolerans kontrolü kritik tıbbi/farmasötik parça imalatçısı.</t>
+        </is>
+      </c>
+      <c r="L988" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> alphacheck -Diabetes Hilfsmittel mit Konzept- CareSens Air CGMS - Berger Med GmbH, tıbbi iğne ve kanül üreticisidir. İğne uçlarının kesim açıları (bevel), dış/iç çapları ve montaj toleranslarının temassız kontrolünde ultra hassas SKANOPT VRE metroloji serisi kullanılabilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" s="2" t="n">
+        <v>988</v>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>Abbott Rapid Diagnostic Germany GmbH</t>
+        </is>
+      </c>
+      <c r="C989" s="2" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="D989" s="2" t="inlineStr"/>
+      <c r="E989" s="2" t="inlineStr">
+        <is>
+          <t>A3 - E6</t>
+        </is>
+      </c>
+      <c r="F989" t="inlineStr">
+        <is>
+          <t>Medikal / Plastik Enjeksiyon</t>
+        </is>
+      </c>
+      <c r="G989" t="inlineStr">
+        <is>
+          <t>EXPOPHARM 2025</t>
+        </is>
+      </c>
+      <c r="H989" t="inlineStr">
+        <is>
+          <t>http://www.globalpointofcare.abbott</t>
+        </is>
+      </c>
+      <c r="I989" t="inlineStr">
+        <is>
+          <t>Tel: 0221271430, 01622180776</t>
+        </is>
+      </c>
+      <c r="J989" s="5" t="inlineStr">
+        <is>
+          <t>Orta Öncelik</t>
+        </is>
+      </c>
+      <c r="K989" s="4" t="inlineStr">
+        <is>
+          <t>Tıbbi ambalaj pompaları, plastik dozaj kapakları, laboratuvar sarf malzemeleri veya teşhis/test stripleri üreten tıbbi plastik enjeksiyon ve montaj firması.</t>
+        </is>
+      </c>
+      <c r="L989" s="4" t="inlineStr">
+        <is>
+          <t>Abbott Rapid Diagnostic Germany GmbH, laboratuvar sarf malzemeleri ve plastik tıbbi ekipmanlar üretmektedir. Plastik pipet uçları, tüpler ve kapakların dairesellik, ovallik ve boyutsal kontrolü için SKANOPT V serisi metroloji çözümleri tavsiye edilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" s="2" t="n">
+        <v>989</v>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CCL Healthcare </t>
+        </is>
+      </c>
+      <c r="C990" s="2" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="D990" s="2" t="inlineStr"/>
+      <c r="E990" s="2" t="inlineStr">
+        <is>
+          <t>A3 IMP - E40</t>
+        </is>
+      </c>
+      <c r="F990" t="inlineStr">
+        <is>
+          <t>Medikal / Plastik Enjeksiyon</t>
+        </is>
+      </c>
+      <c r="G990" t="inlineStr">
+        <is>
+          <t>EXPOPHARM 2025</t>
+        </is>
+      </c>
+      <c r="H990" t="inlineStr">
+        <is>
+          <t>http://www.cclhealthcare.com</t>
+        </is>
+      </c>
+      <c r="I990" t="inlineStr">
+        <is>
+          <t>Tel: 0031615311573, 0033666328993</t>
+        </is>
+      </c>
+      <c r="J990" s="5" t="inlineStr">
+        <is>
+          <t>Orta Öncelik</t>
+        </is>
+      </c>
+      <c r="K990" s="4" t="inlineStr">
+        <is>
+          <t>Tıbbi ambalaj pompaları, plastik dozaj kapakları, laboratuvar sarf malzemeleri veya teşhis/test stripleri üreten tıbbi plastik enjeksiyon ve montaj firması.</t>
+        </is>
+      </c>
+      <c r="L990" s="4" t="inlineStr">
+        <is>
+          <t>CCL Healthcare , laboratuvar sarf malzemeleri ve plastik tıbbi ekipmanlar üretmektedir. Plastik pipet uçları, tüpler ve kapakların dairesellik, ovallik ve boyutsal kontrolü için SKANOPT V serisi metroloji çözümleri tavsiye edilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" s="2" t="n">
+        <v>990</v>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>Dr. Jaglas GmbH</t>
+        </is>
+      </c>
+      <c r="C991" s="2" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="D991" s="2" t="inlineStr"/>
+      <c r="E991" s="2" t="inlineStr">
+        <is>
+          <t>A2 - E44</t>
+        </is>
+      </c>
+      <c r="F991" t="inlineStr">
+        <is>
+          <t>Medikal / Plastik Enjeksiyon</t>
+        </is>
+      </c>
+      <c r="G991" t="inlineStr">
+        <is>
+          <t>EXPOPHARM 2025</t>
+        </is>
+      </c>
+      <c r="H991" t="inlineStr">
+        <is>
+          <t>http://www.dr-jaglas.de</t>
+        </is>
+      </c>
+      <c r="I991" t="inlineStr">
+        <is>
+          <t>Tel: 0049</t>
+        </is>
+      </c>
+      <c r="J991" s="5" t="inlineStr">
+        <is>
+          <t>Orta Öncelik</t>
+        </is>
+      </c>
+      <c r="K991" s="4" t="inlineStr">
+        <is>
+          <t>Tıbbi ambalaj pompaları, plastik dozaj kapakları, laboratuvar sarf malzemeleri veya teşhis/test stripleri üreten tıbbi plastik enjeksiyon ve montaj firması.</t>
+        </is>
+      </c>
+      <c r="L991" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Jaglas GmbH, laboratuvar sarf malzemeleri ve plastik tıbbi ekipmanlar üretmektedir. Plastik pipet uçları, tüpler ve kapakların dairesellik, ovallik ve boyutsal kontrolü için SKANOPT V serisi metroloji çözümleri tavsiye edilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" s="2" t="n">
+        <v>991</v>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>Heaton Deutschland GmbH</t>
+        </is>
+      </c>
+      <c r="C992" s="2" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="D992" s="2" t="inlineStr"/>
+      <c r="E992" s="2" t="inlineStr">
+        <is>
+          <t>A2 - C30 - SCHLOSSALLEE</t>
+        </is>
+      </c>
+      <c r="F992" t="inlineStr">
+        <is>
+          <t>Medikal / Plastik Enjeksiyon</t>
+        </is>
+      </c>
+      <c r="G992" t="inlineStr">
+        <is>
+          <t>EXPOPHARM 2025</t>
+        </is>
+      </c>
+      <c r="H992" t="inlineStr">
+        <is>
+          <t>http://www.gynella.com/de</t>
+        </is>
+      </c>
+      <c r="I992" t="inlineStr">
+        <is>
+          <t>Tel: 004916093414903</t>
+        </is>
+      </c>
+      <c r="J992" s="5" t="inlineStr">
+        <is>
+          <t>Orta Öncelik</t>
+        </is>
+      </c>
+      <c r="K992" s="4" t="inlineStr">
+        <is>
+          <t>Tıbbi ambalaj pompaları, plastik dozaj kapakları, laboratuvar sarf malzemeleri veya teşhis/test stripleri üreten tıbbi plastik enjeksiyon ve montaj firması.</t>
+        </is>
+      </c>
+      <c r="L992" s="4" t="inlineStr">
+        <is>
+          <t>Heaton Deutschland GmbH, laboratuvar sarf malzemeleri ve plastik tıbbi ekipmanlar üretmektedir. Plastik pipet uçları, tüpler ve kapakların dairesellik, ovallik ve boyutsal kontrolü için SKANOPT V serisi metroloji çözümleri tavsiye edilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" s="2" t="n">
+        <v>992</v>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Jiangsu Medomics Medical Technology Co., Ltd</t>
+        </is>
+      </c>
+      <c r="C993" s="2" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="D993" s="2" t="inlineStr"/>
+      <c r="E993" s="2" t="inlineStr">
+        <is>
+          <t>A1 - NC6</t>
+        </is>
+      </c>
+      <c r="F993" t="inlineStr">
+        <is>
+          <t>Medikal / Plastik Enjeksiyon</t>
+        </is>
+      </c>
+      <c r="G993" t="inlineStr">
+        <is>
+          <t>EXPOPHARM 2025</t>
+        </is>
+      </c>
+      <c r="H993" t="inlineStr">
+        <is>
+          <t>https://www.medomics-dx.net/</t>
+        </is>
+      </c>
+      <c r="I993" t="inlineStr">
+        <is>
+          <t>Tel: 008602558601060</t>
+        </is>
+      </c>
+      <c r="J993" s="5" t="inlineStr">
+        <is>
+          <t>Orta Öncelik</t>
+        </is>
+      </c>
+      <c r="K993" s="4" t="inlineStr">
+        <is>
+          <t>Tıbbi ambalaj pompaları, plastik dozaj kapakları, laboratuvar sarf malzemeleri veya teşhis/test stripleri üreten tıbbi plastik enjeksiyon ve montaj firması.</t>
+        </is>
+      </c>
+      <c r="L993" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Jiangsu Medomics Medical Technology Co., Ltd, laboratuvar sarf malzemeleri ve plastik tıbbi ekipmanlar üretmektedir. Plastik pipet uçları, tüpler ve kapakların dairesellik, ovallik ve boyutsal kontrolü için SKANOPT V serisi metroloji çözümleri tavsiye edilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" s="2" t="n">
+        <v>993</v>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>LABORATORIOS BEEMINE SL / The Beemine Lab</t>
+        </is>
+      </c>
+      <c r="C994" s="2" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="D994" s="2" t="inlineStr"/>
+      <c r="E994" s="2" t="inlineStr">
+        <is>
+          <t>A3 - E25</t>
+        </is>
+      </c>
+      <c r="F994" t="inlineStr">
+        <is>
+          <t>Medikal / Plastik Enjeksiyon</t>
+        </is>
+      </c>
+      <c r="G994" t="inlineStr">
+        <is>
+          <t>EXPOPHARM 2025</t>
+        </is>
+      </c>
+      <c r="H994" t="inlineStr">
+        <is>
+          <t>https://thebeeminelab.com/de/</t>
+        </is>
+      </c>
+      <c r="I994" t="inlineStr">
+        <is>
+          <t>Tel: 0034722701808</t>
+        </is>
+      </c>
+      <c r="J994" s="5" t="inlineStr">
+        <is>
+          <t>Orta Öncelik</t>
+        </is>
+      </c>
+      <c r="K994" s="4" t="inlineStr">
+        <is>
+          <t>Tıbbi ambalaj pompaları, plastik dozaj kapakları, laboratuvar sarf malzemeleri veya teşhis/test stripleri üreten tıbbi plastik enjeksiyon ve montaj firması.</t>
+        </is>
+      </c>
+      <c r="L994" s="4" t="inlineStr">
+        <is>
+          <t>LABORATORIOS BEEMINE SL / The Beemine Lab, laboratuvar sarf malzemeleri ve plastik tıbbi ekipmanlar üretmektedir. Plastik pipet uçları, tüpler ve kapakların dairesellik, ovallik ve boyutsal kontrolü için SKANOPT V serisi metroloji çözümleri tavsiye edilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" s="2" t="n">
+        <v>994</v>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>nal von minden GmbH</t>
+        </is>
+      </c>
+      <c r="C995" s="2" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="D995" s="2" t="inlineStr"/>
+      <c r="E995" s="2" t="inlineStr">
+        <is>
+          <t>A2 - E22</t>
+        </is>
+      </c>
+      <c r="F995" t="inlineStr">
+        <is>
+          <t>Medikal / Plastik Enjeksiyon</t>
+        </is>
+      </c>
+      <c r="G995" t="inlineStr">
+        <is>
+          <t>EXPOPHARM 2025</t>
+        </is>
+      </c>
+      <c r="H995" t="inlineStr">
+        <is>
+          <t>https://nal-vonminden.com/</t>
+        </is>
+      </c>
+      <c r="I995" t="inlineStr">
+        <is>
+          <t>Fuar web portalında direkt iletişim bilgisi verilmemiş.</t>
+        </is>
+      </c>
+      <c r="J995" s="5" t="inlineStr">
+        <is>
+          <t>Orta Öncelik</t>
+        </is>
+      </c>
+      <c r="K995" s="4" t="inlineStr">
+        <is>
+          <t>Tıbbi ambalaj pompaları, plastik dozaj kapakları, laboratuvar sarf malzemeleri veya teşhis/test stripleri üreten tıbbi plastik enjeksiyon ve montaj firması.</t>
+        </is>
+      </c>
+      <c r="L995" s="4" t="inlineStr">
+        <is>
+          <t>nal von minden GmbH, laboratuvar sarf malzemeleri ve plastik tıbbi ekipmanlar üretmektedir. Plastik pipet uçları, tüpler ve kapakların dairesellik, ovallik ve boyutsal kontrolü için SKANOPT V serisi metroloji çözümleri tavsiye edilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" s="2" t="n">
+        <v>995</v>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>NOODDIS</t>
+        </is>
+      </c>
+      <c r="C996" s="2" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="D996" s="2" t="inlineStr"/>
+      <c r="E996" s="2" t="inlineStr">
+        <is>
+          <t>A3 - B17</t>
+        </is>
+      </c>
+      <c r="F996" t="inlineStr">
+        <is>
+          <t>Medikal / Hassas Talaşlı İmalat</t>
+        </is>
+      </c>
+      <c r="G996" t="inlineStr">
+        <is>
+          <t>EXPOPHARM 2025</t>
+        </is>
+      </c>
+      <c r="H996" t="inlineStr">
+        <is>
+          <t>https://nooddis.fr/en/liquid-single-dose-preparation-robot-hospital-pharmacy/</t>
+        </is>
+      </c>
+      <c r="I996" t="inlineStr">
+        <is>
+          <t>Fuar web portalında direkt iletişim bilgisi verilmemiş.</t>
+        </is>
+      </c>
+      <c r="J996" s="6" t="inlineStr">
+        <is>
+          <t>Yüksek Öncelik</t>
+        </is>
+      </c>
+      <c r="K996" s="4" t="inlineStr">
+        <is>
+          <t>Hassas iğne, sprey valfleri, insülin kalem iğneleri, lansetler veya ilaç dozaj kovanları üreten, optik metroloji tolerans kontrolü kritik tıbbi/farmasötik parça imalatçısı.</t>
+        </is>
+      </c>
+      <c r="L996" s="4" t="inlineStr">
+        <is>
+          <t>NOODDIS, şırınga, piston ve dozaj kovanları imal etmektedir. Piston yüzey pürüzsüzlüğü, sızdırmazlık kanalları ve boyutsal doğruluğun temassız 0.4 saniye kontrolünde SKANOPT V serisi yüksek verim sağlar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" s="2" t="n">
+        <v>996</v>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>PARI GmbH</t>
+        </is>
+      </c>
+      <c r="C997" s="2" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="D997" s="2" t="inlineStr"/>
+      <c r="E997" s="2" t="inlineStr">
+        <is>
+          <t>A2 - D45</t>
+        </is>
+      </c>
+      <c r="F997" t="inlineStr">
+        <is>
+          <t>Medikal / Hassas Talaşlı İmalat</t>
+        </is>
+      </c>
+      <c r="G997" t="inlineStr">
+        <is>
+          <t>EXPOPHARM 2025</t>
+        </is>
+      </c>
+      <c r="H997" t="inlineStr">
+        <is>
+          <t>http://www.pari.com</t>
+        </is>
+      </c>
+      <c r="I997" t="inlineStr">
+        <is>
+          <t>Fuar web portalında direkt iletişim bilgisi verilmemiş.</t>
+        </is>
+      </c>
+      <c r="J997" s="6" t="inlineStr">
+        <is>
+          <t>Yüksek Öncelik</t>
+        </is>
+      </c>
+      <c r="K997" s="4" t="inlineStr">
+        <is>
+          <t>Hassas iğne, sprey valfleri, insülin kalem iğneleri, lansetler veya ilaç dozaj kovanları üreten, optik metroloji tolerans kontrolü kritik tıbbi/farmasötik parça imalatçısı.</t>
+        </is>
+      </c>
+      <c r="L997" s="4" t="inlineStr">
+        <is>
+          <t>PARI GmbH, dozaj pompaları ve sprey valfleri üretmektedir. Hassas vana parçaları, valf kovanı o-ring kanalları ve nozulların boyutsal ölçümlerinde dikey SKANOPT V serisi kullanımı önerilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" s="2" t="n">
+        <v>997</v>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>Pharmazeutisches Kontroll- und Herstellungslabor GmbH</t>
+        </is>
+      </c>
+      <c r="C998" s="2" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="D998" s="2" t="inlineStr"/>
+      <c r="E998" s="2" t="inlineStr">
+        <is>
+          <t>A2 - B22</t>
+        </is>
+      </c>
+      <c r="F998" t="inlineStr">
+        <is>
+          <t>Medikal / Plastik Enjeksiyon</t>
+        </is>
+      </c>
+      <c r="G998" t="inlineStr">
+        <is>
+          <t>EXPOPHARM 2025</t>
+        </is>
+      </c>
+      <c r="H998" t="inlineStr">
+        <is>
+          <t>https://www.apomix.de</t>
+        </is>
+      </c>
+      <c r="I998" t="inlineStr">
+        <is>
+          <t>Tel: 0049345299780</t>
+        </is>
+      </c>
+      <c r="J998" s="5" t="inlineStr">
+        <is>
+          <t>Orta Öncelik</t>
+        </is>
+      </c>
+      <c r="K998" s="4" t="inlineStr">
+        <is>
+          <t>Tıbbi ambalaj pompaları, plastik dozaj kapakları, laboratuvar sarf malzemeleri veya teşhis/test stripleri üreten tıbbi plastik enjeksiyon ve montaj firması.</t>
+        </is>
+      </c>
+      <c r="L998" s="4" t="inlineStr">
+        <is>
+          <t>Pharmazeutisches Kontroll- und Herstellungslabor GmbH, laboratuvar sarf malzemeleri ve plastik tıbbi ekipmanlar üretmektedir. Plastik pipet uçları, tüpler ve kapakların dairesellik, ovallik ve boyutsal kontrolü için SKANOPT V serisi metroloji çözümleri tavsiye edilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" s="2" t="n">
+        <v>998</v>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>SKAITOS KOMPIUTERIŲ SERVISAS UAB</t>
+        </is>
+      </c>
+      <c r="C999" s="2" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="D999" s="2" t="inlineStr"/>
+      <c r="E999" s="2" t="inlineStr">
+        <is>
+          <t>A1 - A29</t>
+        </is>
+      </c>
+      <c r="F999" t="inlineStr">
+        <is>
+          <t>Medikal / Plastik Enjeksiyon</t>
+        </is>
+      </c>
+      <c r="G999" t="inlineStr">
+        <is>
+          <t>EXPOPHARM 2025</t>
+        </is>
+      </c>
+      <c r="H999" t="inlineStr">
+        <is>
+          <t>http://www.sks.lt</t>
+        </is>
+      </c>
+      <c r="I999" t="inlineStr">
+        <is>
+          <t>Tel: 00370370330220, 0037065093764, 0037065509449</t>
+        </is>
+      </c>
+      <c r="J999" s="5" t="inlineStr">
+        <is>
+          <t>Orta Öncelik</t>
+        </is>
+      </c>
+      <c r="K999" s="4" t="inlineStr">
+        <is>
+          <t>Tıbbi ambalaj pompaları, plastik dozaj kapakları, laboratuvar sarf malzemeleri veya teşhis/test stripleri üreten tıbbi plastik enjeksiyon ve montaj firması.</t>
+        </is>
+      </c>
+      <c r="L999" s="4" t="inlineStr">
+        <is>
+          <t>SKAITOS KOMPIUTERIŲ SERVISAS UAB, laboratuvar sarf malzemeleri ve plastik tıbbi ekipmanlar üretmektedir. Plastik pipet uçları, tüpler ve kapakların dairesellik, ovallik ve boyutsal kontrolü için SKANOPT V serisi metroloji çözümleri tavsiye edilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="2" t="n">
+        <v>999</v>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>WEPA Apothekenbedarf GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="C1000" s="2" t="inlineStr">
+        <is>
+          <t>Almanya</t>
+        </is>
+      </c>
+      <c r="D1000" s="2" t="inlineStr"/>
+      <c r="E1000" s="2" t="inlineStr">
+        <is>
+          <t>A2 - C4</t>
+        </is>
+      </c>
+      <c r="F1000" t="inlineStr">
+        <is>
+          <t>Medikal / Plastik Enjeksiyon</t>
+        </is>
+      </c>
+      <c r="G1000" t="inlineStr">
+        <is>
+          <t>EXPOPHARM 2025</t>
+        </is>
+      </c>
+      <c r="H1000" t="inlineStr">
+        <is>
+          <t>https://www.wepa-apothekenbedarf.de/</t>
+        </is>
+      </c>
+      <c r="I1000" t="inlineStr">
+        <is>
+          <t>Tel: 026241070</t>
+        </is>
+      </c>
+      <c r="J1000" s="5" t="inlineStr">
+        <is>
+          <t>Orta Öncelik</t>
+        </is>
+      </c>
+      <c r="K1000" s="4" t="inlineStr">
+        <is>
+          <t>Tıbbi ambalaj pompaları, plastik dozaj kapakları, laboratuvar sarf malzemeleri veya teşhis/test stripleri üreten tıbbi plastik enjeksiyon ve montaj firması.</t>
+        </is>
+      </c>
+      <c r="L1000" s="4" t="inlineStr">
+        <is>
+          <t>WEPA Apothekenbedarf GmbH &amp; Co. KG, laboratuvar sarf malzemeleri ve plastik tıbbi ekipmanlar üretmektedir. Plastik pipet uçları, tüpler ve kapakların dairesellik, ovallik ve boyutsal kontrolü için SKANOPT V serisi metroloji çözümleri tavsiye edilir.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L987"/>
+  <autoFilter ref="A1:L1000"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>